<commit_message>
Test local pour Moissonnage
</commit_message>
<xml_diff>
--- a/donnees/AAD_dataframe_partial_inventory.xlsx
+++ b/donnees/AAD_dataframe_partial_inventory.xlsx
@@ -20,16 +20,13 @@
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
     <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -40,7 +37,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -48,21 +45,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -433,42 +421,42 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>ID</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>NUM_URL</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>HTML_URL</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>HTML_ACCESS</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>HTML_ADATE</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>PDF_URL</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>PDF_ACCESS</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>PDF_ADATE</t>
         </is>
@@ -493,8 +481,8 @@
       <c r="D2" t="b">
         <v>1</v>
       </c>
-      <c r="E2" s="2" t="n">
-        <v>46325.79541875009</v>
+      <c r="E2" s="1" t="n">
+        <v>46326.23388888952</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -504,8 +492,8 @@
       <c r="G2" t="b">
         <v>1</v>
       </c>
-      <c r="H2" s="2" t="n">
-        <v>46325.7962044034</v>
+      <c r="H2" s="1" t="n">
+        <v>46326.23454772711</v>
       </c>
     </row>
     <row r="3">
@@ -527,8 +515,8 @@
       <c r="D3" t="b">
         <v>1</v>
       </c>
-      <c r="E3" s="2" t="n">
-        <v>46325.79545746921</v>
+      <c r="E3" s="1" t="n">
+        <v>46326.23393265956</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -538,8 +526,8 @@
       <c r="G3" t="b">
         <v>1</v>
       </c>
-      <c r="H3" s="2" t="n">
-        <v>46325.79625200819</v>
+      <c r="H3" s="1" t="n">
+        <v>46326.23459545021</v>
       </c>
     </row>
     <row r="4">
@@ -561,8 +549,8 @@
       <c r="D4" t="b">
         <v>1</v>
       </c>
-      <c r="E4" s="2" t="n">
-        <v>46325.79549614175</v>
+      <c r="E4" s="1" t="n">
+        <v>46326.23397532698</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -572,8 +560,8 @@
       <c r="G4" t="b">
         <v>1</v>
       </c>
-      <c r="H4" s="2" t="n">
-        <v>46325.79629690829</v>
+      <c r="H4" s="1" t="n">
+        <v>46326.23464233411</v>
       </c>
     </row>
     <row r="5">
@@ -595,8 +583,8 @@
       <c r="D5" t="b">
         <v>1</v>
       </c>
-      <c r="E5" s="2" t="n">
-        <v>46325.79553448276</v>
+      <c r="E5" s="1" t="n">
+        <v>46326.2340177203</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
@@ -606,8 +594,8 @@
       <c r="G5" t="b">
         <v>1</v>
       </c>
-      <c r="H5" s="2" t="n">
-        <v>46325.79634438726</v>
+      <c r="H5" s="1" t="n">
+        <v>46326.23468988224</v>
       </c>
     </row>
     <row r="6">
@@ -629,8 +617,8 @@
       <c r="D6" t="b">
         <v>1</v>
       </c>
-      <c r="E6" s="2" t="n">
-        <v>46325.79557204984</v>
+      <c r="E6" s="1" t="n">
+        <v>46326.23405973586</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
@@ -640,8 +628,8 @@
       <c r="G6" t="b">
         <v>1</v>
       </c>
-      <c r="H6" s="2" t="n">
-        <v>46325.79639681755</v>
+      <c r="H6" s="1" t="n">
+        <v>46326.23473960831</v>
       </c>
     </row>
     <row r="7">
@@ -663,8 +651,8 @@
       <c r="D7" t="b">
         <v>1</v>
       </c>
-      <c r="E7" s="2" t="n">
-        <v>46325.79561013265</v>
+      <c r="E7" s="1" t="n">
+        <v>46326.23410400502</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
@@ -674,8 +662,8 @@
       <c r="G7" t="b">
         <v>1</v>
       </c>
-      <c r="H7" s="2" t="n">
-        <v>46325.79644181948</v>
+      <c r="H7" s="1" t="n">
+        <v>46326.23479690475</v>
       </c>
     </row>
     <row r="8">
@@ -697,8 +685,8 @@
       <c r="D8" t="b">
         <v>1</v>
       </c>
-      <c r="E8" s="2" t="n">
-        <v>46325.79564886904</v>
+      <c r="E8" s="1" t="n">
+        <v>46326.23414795622</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
@@ -708,8 +696,8 @@
       <c r="G8" t="b">
         <v>1</v>
       </c>
-      <c r="H8" s="2" t="n">
-        <v>46325.79648666089</v>
+      <c r="H8" s="1" t="n">
+        <v>46326.23484262075</v>
       </c>
     </row>
     <row r="9">
@@ -731,8 +719,8 @@
       <c r="D9" t="b">
         <v>1</v>
       </c>
-      <c r="E9" s="2" t="n">
-        <v>46325.7956875547</v>
+      <c r="E9" s="1" t="n">
+        <v>46326.23419067674</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
@@ -742,8 +730,8 @@
       <c r="G9" t="b">
         <v>1</v>
       </c>
-      <c r="H9" s="2" t="n">
-        <v>46325.79653308009</v>
+      <c r="H9" s="1" t="n">
+        <v>46326.23488962296</v>
       </c>
     </row>
     <row r="10">
@@ -765,8 +753,8 @@
       <c r="D10" t="b">
         <v>1</v>
       </c>
-      <c r="E10" s="2" t="n">
-        <v>46325.79573376988</v>
+      <c r="E10" s="1" t="n">
+        <v>46326.23423369138</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
@@ -776,8 +764,8 @@
       <c r="G10" t="b">
         <v>1</v>
       </c>
-      <c r="H10" s="2" t="n">
-        <v>46325.7965777096</v>
+      <c r="H10" s="1" t="n">
+        <v>46326.23493504185</v>
       </c>
     </row>
     <row r="11">
@@ -799,8 +787,8 @@
       <c r="D11" t="b">
         <v>1</v>
       </c>
-      <c r="E11" s="2" t="n">
-        <v>46325.79577245773</v>
+      <c r="E11" s="1" t="n">
+        <v>46326.23427615866</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
@@ -810,8 +798,8 @@
       <c r="G11" t="b">
         <v>1</v>
       </c>
-      <c r="H11" s="2" t="n">
-        <v>46325.79662361104</v>
+      <c r="H11" s="1" t="n">
+        <v>46326.23498261914</v>
       </c>
     </row>
     <row r="12">
@@ -833,8 +821,8 @@
       <c r="D12" t="b">
         <v>1</v>
       </c>
-      <c r="E12" s="2" t="n">
-        <v>46325.79581855965</v>
+      <c r="E12" s="1" t="n">
+        <v>46326.23431863997</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
@@ -844,8 +832,8 @@
       <c r="G12" t="b">
         <v>1</v>
       </c>
-      <c r="H12" s="2" t="n">
-        <v>46325.79667135625</v>
+      <c r="H12" s="1" t="n">
+        <v>46326.23503054569</v>
       </c>
     </row>
     <row r="13">
@@ -867,8 +855,8 @@
       <c r="D13" t="b">
         <v>1</v>
       </c>
-      <c r="E13" s="2" t="n">
-        <v>46325.79585720717</v>
+      <c r="E13" s="1" t="n">
+        <v>46326.23436257238</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
@@ -878,8 +866,8 @@
       <c r="G13" t="b">
         <v>1</v>
       </c>
-      <c r="H13" s="2" t="n">
-        <v>46325.79671654698</v>
+      <c r="H13" s="1" t="n">
+        <v>46326.23507804694</v>
       </c>
     </row>
     <row r="14">
@@ -901,8 +889,8 @@
       <c r="D14" t="b">
         <v>1</v>
       </c>
-      <c r="E14" s="2" t="n">
-        <v>46325.79589488618</v>
+      <c r="E14" s="1" t="n">
+        <v>46326.23440513852</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
@@ -912,8 +900,8 @@
       <c r="G14" t="b">
         <v>1</v>
       </c>
-      <c r="H14" s="2" t="n">
-        <v>46325.79676138233</v>
+      <c r="H14" s="1" t="n">
+        <v>46326.23512498187</v>
       </c>
     </row>
     <row r="15">
@@ -935,8 +923,8 @@
       <c r="D15" t="b">
         <v>1</v>
       </c>
-      <c r="E15" s="2" t="n">
-        <v>46325.79593357358</v>
+      <c r="E15" s="1" t="n">
+        <v>46326.2344473987</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
@@ -946,8 +934,8 @@
       <c r="G15" t="b">
         <v>0</v>
       </c>
-      <c r="H15" s="2" t="n">
-        <v>46325.79680049941</v>
+      <c r="H15" s="1" t="n">
+        <v>46326.23516293192</v>
       </c>
     </row>
   </sheetData>

</xml_diff>